<commit_message>
Update daily rolling forecast for 2026-09-12
</commit_message>
<xml_diff>
--- a/data/2026_09/snapshots/2026_09_12/dashboard_v3.xlsx
+++ b/data/2026_09/snapshots/2026_09_12/dashboard_v3.xlsx
@@ -491,16 +491,16 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>19029634</v>
+        <v>19035025</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>19752670</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>-723036</v>
+        <v>-717645</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-3.7</v>
+        <v>-3.6</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -515,16 +515,16 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>20987186</v>
+        <v>20992577</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>19752670</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1234516</v>
+        <v>1239907</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -539,16 +539,16 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>12750483</v>
+        <v>12755875</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>13693510</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>-943027</v>
+        <v>-937635</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-6.9</v>
+        <v>-6.8</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -635,16 +635,16 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>1358</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-1.6</v>
+        <v>-1.5</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -707,16 +707,16 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>751</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>26.4</v>
+        <v>26.5</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -731,16 +731,16 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>380</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>4.7</v>
+        <v>5.3</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>現時点着地見込み 1,903万円は前年同月 1,975万円を下回る見込み（前年差 ▲72万・-3.7%）。一方、通常営業ベース 2,099万円は前年を上回る（+6.2%）。差 ▲196万は通常営業ベースとの差であり、自費売上化と他曜日充足で埋められるかが焦点。</t>
+          <t>現時点着地見込み 1,904万円は前年同月 1,975万円を下回る見込み（前年差 ▲72万・-3.6%）。一方、通常営業ベース 2,099万円は前年を上回る（+6.3%）。差 ▲196万は通常営業ベースとの差であり、自費売上化と他曜日充足で埋められるかが焦点。</t>
         </is>
       </c>
     </row>

</xml_diff>